<commit_message>
Finished intra truck logic
Signed-off-by: Bhavya <bhavya_b@mit.edu>
</commit_message>
<xml_diff>
--- a/Model_Stops.xlsx
+++ b/Model_Stops.xlsx
@@ -8540,7 +8540,7 @@
         <v>-81.02224330555725</v>
       </c>
       <c r="E267" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F267" t="n">
         <v>1</v>
@@ -27770,7 +27770,7 @@
         <v>-85.18380671739578</v>
       </c>
       <c r="E899" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="F899" t="n">
         <v>1</v>
@@ -28195,7 +28195,9 @@
       <c r="D913" t="n">
         <v>-85.27912443245411</v>
       </c>
-      <c r="E913" t="inlineStr"/>
+      <c r="E913" t="n">
+        <v>60</v>
+      </c>
       <c r="F913" t="n">
         <v>1</v>
       </c>
@@ -33676,7 +33678,7 @@
         <v>-85.263639</v>
       </c>
       <c r="E1093" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F1093" t="n">
         <v>1</v>
@@ -33707,7 +33709,7 @@
         <v>-85.263639</v>
       </c>
       <c r="E1094" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F1094" t="n">
         <v>1</v>
@@ -37042,7 +37044,7 @@
         <v>-84.66229338276864</v>
       </c>
       <c r="E1203" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F1203" t="n">
         <v>1</v>
@@ -37073,7 +37075,7 @@
         <v>-84.66229338276864</v>
       </c>
       <c r="E1204" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F1204" t="n">
         <v>1</v>
@@ -37799,7 +37801,7 @@
         <v>-88.3285571423626</v>
       </c>
       <c r="E1228" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F1228" t="n">
         <v>3</v>
@@ -38566,7 +38568,7 @@
         <v>-86.16333313624573</v>
       </c>
       <c r="E1253" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F1253" t="n">
         <v>1</v>
@@ -38597,7 +38599,7 @@
         <v>-86.16333313624573</v>
       </c>
       <c r="E1254" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F1254" t="n">
         <v>1</v>
@@ -49605,7 +49607,7 @@
         <v>-82.0615740821743</v>
       </c>
       <c r="E1616" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F1616" t="n">
         <v>1</v>
@@ -49681,169 +49683,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A9D0198779F64D4583CB0D0F5191282D" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="265535fc1b2f34fa73935fce8401c032">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6a14bfa0-ee12-46b7-910d-7c55fe0c806e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="24633c4a450fef35b4745f60ee9eccd8" ns2:_="">
-    <xsd:import namespace="6a14bfa0-ee12-46b7-910d-7c55fe0c806e"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="6a14bfa0-ee12-46b7-910d-7c55fe0c806e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECCB8FE3-6E53-49AC-9ED4-983ECE52F2C6}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{622133F4-62FD-4FEC-8170-C29CBE10FE2C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B8F2282-B03E-446F-B763-B91E767D940E}"/>
 </file>
</xml_diff>